<commit_message>
Created main and export_to_excel master_to_pandas.ipynb: -removed old excel export functions
</commit_message>
<xml_diff>
--- a/Program/master_lines.xlsx
+++ b/Program/master_lines.xlsx
@@ -7,10 +7,10 @@
     <workbookView visibility="visible" minimized="0" showHorizontalScroll="1" showVerticalScroll="1" showSheetTabs="1" tabRatio="600" firstSheet="0" activeTab="0" autoFilterDateGrouping="1"/>
   </bookViews>
   <sheets>
-    <sheet name="Master Lines" sheetId="1" state="visible" r:id="rId1"/>
+    <sheet name="Lines" sheetId="1" state="visible" r:id="rId1"/>
   </sheets>
   <definedNames>
-    <definedName name="_xlnm._FilterDatabase" localSheetId="0" hidden="1">'Master Lines'!$A$1:$BK$17</definedName>
+    <definedName name="_xlnm._FilterDatabase" localSheetId="0" hidden="1">'Lines'!$A$1:$BL$17</definedName>
   </definedNames>
   <calcPr calcId="124519" fullCalcOnLoad="1"/>
 </workbook>
@@ -68,19 +68,19 @@
       <diagonal/>
     </border>
     <border>
-      <left/>
-      <right style="thick">
+      <left style="thick">
         <color rgb="FF4169E1"/>
-      </right>
+      </left>
+      <right/>
       <top/>
       <bottom/>
       <diagonal/>
     </border>
     <border>
-      <left style="thick">
+      <left/>
+      <right style="thick">
         <color rgb="FF4169E1"/>
-      </left>
-      <right/>
+      </right>
       <top/>
       <bottom/>
       <diagonal/>
@@ -109,13 +109,13 @@
     <xf numFmtId="0" fontId="0" fillId="2" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="center" vertical="center" wrapText="1"/>
     </xf>
-    <xf numFmtId="0" fontId="0" fillId="2" borderId="4" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+    <xf numFmtId="0" fontId="0" fillId="2" borderId="3" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="center" vertical="center" wrapText="1"/>
     </xf>
     <xf numFmtId="0" fontId="0" fillId="2" borderId="2" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="center" vertical="center" wrapText="1"/>
     </xf>
-    <xf numFmtId="0" fontId="0" fillId="2" borderId="3" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+    <xf numFmtId="0" fontId="0" fillId="2" borderId="4" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="center" vertical="center" wrapText="1"/>
     </xf>
     <xf numFmtId="0" fontId="0" fillId="2" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
@@ -198,9 +198,9 @@
 </file>
 
 <file path=xl/tables/table1.xml><?xml version="1.0" encoding="utf-8"?>
-<table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" id="1" name="MasterLinesTable" displayName="MasterLinesTable" ref="A1:BK17" headerRowCount="1">
-  <autoFilter ref="A1:BK17"/>
-  <tableColumns count="63">
+<table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" id="1" name="LinesTable" displayName="LinesTable" ref="A1:BL17" headerRowCount="1">
+  <autoFilter ref="A1:BL17"/>
+  <tableColumns count="64">
     <tableColumn id="1" name="Line Number"/>
     <tableColumn id="2" name="Extra Vacation Days"/>
     <tableColumn id="3" name="Sun, May 21"/>
@@ -264,6 +264,7 @@
     <tableColumn id="61" name="Total DO"/>
     <tableColumn id="62" name="% tickets paid"/>
     <tableColumn id="63" name="Premium"/>
+    <tableColumn id="64" name="Start bid off"/>
   </tableColumns>
   <tableStyleInfo name="TableStyleLight9" showFirstColumn="0" showLastColumn="0" showRowStripes="1" showColumnStripes="0"/>
 </table>
@@ -558,7 +559,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:BK17"/>
+  <dimension ref="A1:BL17"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="13" customWidth="1" min="1" max="1"/>
@@ -624,6 +625,7 @@
     <col width="10" customWidth="1" min="61" max="61"/>
     <col width="16" customWidth="1" min="62" max="62"/>
     <col width="9" customWidth="1" min="63" max="63"/>
+    <col width="15" customWidth="1" min="64" max="64"/>
   </cols>
   <sheetData>
     <row r="1" ht="36" customHeight="1">
@@ -637,7 +639,7 @@
           <t>Extra Vacation Days</t>
         </is>
       </c>
-      <c r="C1" s="2" t="inlineStr">
+      <c r="C1" s="1" t="inlineStr">
         <is>
           <t>Sun, May 21</t>
         </is>
@@ -692,7 +694,7 @@
           <t>Wed, May 31</t>
         </is>
       </c>
-      <c r="N1" s="3" t="inlineStr">
+      <c r="N1" s="2" t="inlineStr">
         <is>
           <t>Thu, Jun 1</t>
         </is>
@@ -727,7 +729,7 @@
           <t>Wed, Jun 7</t>
         </is>
       </c>
-      <c r="U1" s="2" t="inlineStr">
+      <c r="U1" s="3" t="inlineStr">
         <is>
           <t>Thu, Jun 8</t>
         </is>
@@ -940,6 +942,11 @@
       <c r="BK1" s="1" t="inlineStr">
         <is>
           <t>Premium</t>
+        </is>
+      </c>
+      <c r="BL1" s="1" t="inlineStr">
+        <is>
+          <t>Start bid off</t>
         </is>
       </c>
     </row>
@@ -950,7 +957,7 @@
       <c r="B2" t="n">
         <v>7</v>
       </c>
-      <c r="C2" s="2" t="inlineStr"/>
+      <c r="C2" s="1" t="inlineStr"/>
       <c r="D2" s="1" t="inlineStr"/>
       <c r="E2" s="1" t="inlineStr"/>
       <c r="F2" s="1" t="inlineStr"/>
@@ -996,7 +1003,7 @@
       <c r="R2" s="1" t="inlineStr"/>
       <c r="S2" s="1" t="inlineStr"/>
       <c r="T2" s="1" t="inlineStr"/>
-      <c r="U2" s="2" t="inlineStr"/>
+      <c r="U2" s="3" t="inlineStr"/>
       <c r="V2" s="1" t="inlineStr"/>
       <c r="W2" s="1" t="inlineStr"/>
       <c r="X2" s="6" t="inlineStr">
@@ -1131,6 +1138,9 @@
       <c r="BK2" t="n">
         <v>0</v>
       </c>
+      <c r="BL2" t="n">
+        <v>7</v>
+      </c>
     </row>
     <row r="3" ht="28" customHeight="1">
       <c r="A3" t="n">
@@ -1139,7 +1149,7 @@
       <c r="B3" t="n">
         <v>7</v>
       </c>
-      <c r="C3" s="2" t="inlineStr"/>
+      <c r="C3" s="1" t="inlineStr"/>
       <c r="D3" s="1" t="inlineStr"/>
       <c r="E3" s="1" t="inlineStr"/>
       <c r="F3" s="1" t="inlineStr"/>
@@ -1185,7 +1195,7 @@
       <c r="R3" s="1" t="inlineStr"/>
       <c r="S3" s="1" t="inlineStr"/>
       <c r="T3" s="1" t="inlineStr"/>
-      <c r="U3" s="2" t="inlineStr"/>
+      <c r="U3" s="3" t="inlineStr"/>
       <c r="V3" s="1" t="inlineStr"/>
       <c r="W3" s="1" t="inlineStr"/>
       <c r="X3" s="6" t="inlineStr">
@@ -1320,6 +1330,9 @@
       <c r="BK3" t="n">
         <v>0</v>
       </c>
+      <c r="BL3" t="n">
+        <v>7</v>
+      </c>
     </row>
     <row r="4" ht="28" customHeight="1">
       <c r="A4" t="n">
@@ -1328,7 +1341,7 @@
       <c r="B4" t="n">
         <v>2</v>
       </c>
-      <c r="C4" s="2" t="inlineStr"/>
+      <c r="C4" s="1" t="inlineStr"/>
       <c r="D4" s="1" t="inlineStr"/>
       <c r="E4" s="6" t="inlineStr">
         <is>
@@ -1359,7 +1372,7 @@
       <c r="K4" s="1" t="inlineStr"/>
       <c r="L4" s="1" t="inlineStr"/>
       <c r="M4" s="1" t="inlineStr"/>
-      <c r="N4" s="3" t="inlineStr"/>
+      <c r="N4" s="2" t="inlineStr"/>
       <c r="O4" s="1" t="inlineStr"/>
       <c r="P4" s="1" t="inlineStr"/>
       <c r="Q4" s="1" t="inlineStr"/>
@@ -1489,6 +1502,9 @@
       <c r="BK4" t="n">
         <v>0</v>
       </c>
+      <c r="BL4" t="n">
+        <v>2</v>
+      </c>
     </row>
     <row r="5" ht="28" customHeight="1">
       <c r="A5" t="n">
@@ -1497,7 +1513,7 @@
       <c r="B5" t="n">
         <v>2</v>
       </c>
-      <c r="C5" s="2" t="inlineStr"/>
+      <c r="C5" s="1" t="inlineStr"/>
       <c r="D5" s="1" t="inlineStr"/>
       <c r="E5" s="6" t="inlineStr">
         <is>
@@ -1662,6 +1678,9 @@
       <c r="BK5" t="n">
         <v>0</v>
       </c>
+      <c r="BL5" t="n">
+        <v>2</v>
+      </c>
     </row>
     <row r="6" ht="28" customHeight="1">
       <c r="A6" t="n">
@@ -1670,7 +1689,7 @@
       <c r="B6" t="n">
         <v>2</v>
       </c>
-      <c r="C6" s="2" t="inlineStr"/>
+      <c r="C6" s="1" t="inlineStr"/>
       <c r="D6" s="1" t="inlineStr"/>
       <c r="E6" s="6" t="inlineStr">
         <is>
@@ -1724,7 +1743,7 @@
       <c r="R6" s="1" t="inlineStr"/>
       <c r="S6" s="1" t="inlineStr"/>
       <c r="T6" s="1" t="inlineStr"/>
-      <c r="U6" s="2" t="inlineStr"/>
+      <c r="U6" s="3" t="inlineStr"/>
       <c r="V6" s="1" t="inlineStr"/>
       <c r="W6" s="1" t="inlineStr"/>
       <c r="X6" s="1" t="inlineStr"/>
@@ -1851,6 +1870,9 @@
       <c r="BK6" t="n">
         <v>0</v>
       </c>
+      <c r="BL6" t="n">
+        <v>2</v>
+      </c>
     </row>
     <row r="7" ht="28" customHeight="1">
       <c r="A7" t="n">
@@ -1859,7 +1881,7 @@
       <c r="B7" t="n">
         <v>1</v>
       </c>
-      <c r="C7" s="2" t="inlineStr"/>
+      <c r="C7" s="1" t="inlineStr"/>
       <c r="D7" s="6" t="inlineStr">
         <is>
           <t>RA</t>
@@ -2040,6 +2062,9 @@
       <c r="BK7" t="n">
         <v>0</v>
       </c>
+      <c r="BL7" t="n">
+        <v>1</v>
+      </c>
     </row>
     <row r="8" ht="28" customHeight="1">
       <c r="A8" t="n">
@@ -2048,7 +2073,7 @@
       <c r="B8" t="n">
         <v>0</v>
       </c>
-      <c r="C8" s="9" t="inlineStr">
+      <c r="C8" s="6" t="inlineStr">
         <is>
           <t>{291SDF-</t>
         </is>
@@ -2083,14 +2108,14 @@
       <c r="K8" s="1" t="inlineStr"/>
       <c r="L8" s="1" t="inlineStr"/>
       <c r="M8" s="1" t="inlineStr"/>
-      <c r="N8" s="3" t="inlineStr"/>
+      <c r="N8" s="2" t="inlineStr"/>
       <c r="O8" s="1" t="inlineStr"/>
       <c r="P8" s="1" t="inlineStr"/>
       <c r="Q8" s="1" t="inlineStr"/>
       <c r="R8" s="1" t="inlineStr"/>
       <c r="S8" s="1" t="inlineStr"/>
       <c r="T8" s="1" t="inlineStr"/>
-      <c r="U8" s="2" t="inlineStr"/>
+      <c r="U8" s="3" t="inlineStr"/>
       <c r="V8" s="1" t="inlineStr"/>
       <c r="W8" s="1" t="inlineStr"/>
       <c r="X8" s="6" t="inlineStr">
@@ -2225,6 +2250,9 @@
       <c r="BK8" t="n">
         <v>0</v>
       </c>
+      <c r="BL8" t="n">
+        <v>0</v>
+      </c>
     </row>
     <row r="9" ht="28" customHeight="1">
       <c r="A9" t="n">
@@ -2233,7 +2261,7 @@
       <c r="B9" t="n">
         <v>0</v>
       </c>
-      <c r="C9" s="9" t="inlineStr">
+      <c r="C9" s="6" t="inlineStr">
         <is>
           <t>{307SDF-</t>
         </is>
@@ -2272,7 +2300,7 @@
       <c r="K9" s="1" t="inlineStr"/>
       <c r="L9" s="1" t="inlineStr"/>
       <c r="M9" s="1" t="inlineStr"/>
-      <c r="N9" s="3" t="inlineStr"/>
+      <c r="N9" s="2" t="inlineStr"/>
       <c r="O9" s="1" t="inlineStr"/>
       <c r="P9" s="1" t="inlineStr"/>
       <c r="Q9" s="6" t="inlineStr">
@@ -2418,6 +2446,9 @@
       <c r="BK9" t="n">
         <v>0</v>
       </c>
+      <c r="BL9" t="n">
+        <v>0</v>
+      </c>
     </row>
     <row r="10" ht="28" customHeight="1">
       <c r="A10" t="n">
@@ -2426,7 +2457,7 @@
       <c r="B10" t="n">
         <v>0</v>
       </c>
-      <c r="C10" s="9" t="inlineStr">
+      <c r="C10" s="6" t="inlineStr">
         <is>
           <t>{395SDF-(DH DL)[ATL25.5]</t>
         </is>
@@ -2469,14 +2500,14 @@
       <c r="K10" s="1" t="inlineStr"/>
       <c r="L10" s="1" t="inlineStr"/>
       <c r="M10" s="1" t="inlineStr"/>
-      <c r="N10" s="3" t="inlineStr"/>
+      <c r="N10" s="2" t="inlineStr"/>
       <c r="O10" s="1" t="inlineStr"/>
       <c r="P10" s="1" t="inlineStr"/>
       <c r="Q10" s="1" t="inlineStr"/>
       <c r="R10" s="1" t="inlineStr"/>
       <c r="S10" s="1" t="inlineStr"/>
       <c r="T10" s="1" t="inlineStr"/>
-      <c r="U10" s="2" t="inlineStr"/>
+      <c r="U10" s="3" t="inlineStr"/>
       <c r="V10" s="1" t="inlineStr"/>
       <c r="W10" s="1" t="inlineStr"/>
       <c r="X10" s="6" t="inlineStr">
@@ -2661,6 +2692,9 @@
         <v>75</v>
       </c>
       <c r="BK10" t="n">
+        <v>0</v>
+      </c>
+      <c r="BL10" t="n">
         <v>0</v>
       </c>
     </row>
@@ -2671,7 +2705,7 @@
       <c r="B11" t="n">
         <v>0</v>
       </c>
-      <c r="C11" s="9" t="inlineStr">
+      <c r="C11" s="6" t="inlineStr">
         <is>
           <t>VTO</t>
         </is>
@@ -2900,6 +2934,9 @@
       <c r="BK11" t="n">
         <v>439</v>
       </c>
+      <c r="BL11" t="n">
+        <v>0</v>
+      </c>
     </row>
     <row r="12" ht="28" customHeight="1">
       <c r="A12" t="n">
@@ -2908,7 +2945,7 @@
       <c r="B12" t="n">
         <v>0</v>
       </c>
-      <c r="C12" s="9" t="inlineStr">
+      <c r="C12" s="6" t="inlineStr">
         <is>
           <t>VTO</t>
         </is>
@@ -3199,6 +3236,9 @@
         <v>0</v>
       </c>
       <c r="BK12" t="n">
+        <v>0</v>
+      </c>
+      <c r="BL12" t="n">
         <v>0</v>
       </c>
     </row>
@@ -3209,7 +3249,7 @@
       <c r="B13" t="n">
         <v>0</v>
       </c>
-      <c r="C13" s="9" t="inlineStr">
+      <c r="C13" s="6" t="inlineStr">
         <is>
           <t>RB</t>
         </is>
@@ -3263,7 +3303,7 @@
       <c r="R13" s="1" t="inlineStr"/>
       <c r="S13" s="1" t="inlineStr"/>
       <c r="T13" s="1" t="inlineStr"/>
-      <c r="U13" s="2" t="inlineStr"/>
+      <c r="U13" s="3" t="inlineStr"/>
       <c r="V13" s="1" t="inlineStr"/>
       <c r="W13" s="1" t="inlineStr"/>
       <c r="X13" s="6" t="inlineStr">
@@ -3390,6 +3430,9 @@
       <c r="BK13" t="n">
         <v>0</v>
       </c>
+      <c r="BL13" t="n">
+        <v>0</v>
+      </c>
     </row>
     <row r="14" ht="28" customHeight="1">
       <c r="A14" t="n">
@@ -3398,7 +3441,7 @@
       <c r="B14" t="n">
         <v>0</v>
       </c>
-      <c r="C14" s="9" t="inlineStr">
+      <c r="C14" s="6" t="inlineStr">
         <is>
           <t>SB</t>
         </is>
@@ -3437,7 +3480,7 @@
       <c r="K14" s="1" t="inlineStr"/>
       <c r="L14" s="1" t="inlineStr"/>
       <c r="M14" s="1" t="inlineStr"/>
-      <c r="N14" s="3" t="inlineStr"/>
+      <c r="N14" s="2" t="inlineStr"/>
       <c r="O14" s="1" t="inlineStr"/>
       <c r="P14" s="1" t="inlineStr"/>
       <c r="Q14" s="6" t="inlineStr">
@@ -3579,6 +3622,9 @@
       <c r="BK14" t="n">
         <v>0</v>
       </c>
+      <c r="BL14" t="n">
+        <v>0</v>
+      </c>
     </row>
     <row r="15" ht="28" customHeight="1">
       <c r="A15" t="n">
@@ -3587,7 +3633,7 @@
       <c r="B15" t="n">
         <v>0</v>
       </c>
-      <c r="C15" s="9" t="inlineStr">
+      <c r="C15" s="6" t="inlineStr">
         <is>
           <t>SA</t>
         </is>
@@ -3626,7 +3672,7 @@
       <c r="K15" s="1" t="inlineStr"/>
       <c r="L15" s="1" t="inlineStr"/>
       <c r="M15" s="1" t="inlineStr"/>
-      <c r="N15" s="3" t="inlineStr"/>
+      <c r="N15" s="2" t="inlineStr"/>
       <c r="O15" s="1" t="inlineStr"/>
       <c r="P15" s="1" t="inlineStr"/>
       <c r="Q15" s="6" t="inlineStr">
@@ -3768,6 +3814,9 @@
       <c r="BK15" t="n">
         <v>0</v>
       </c>
+      <c r="BL15" t="n">
+        <v>0</v>
+      </c>
     </row>
     <row r="16" ht="28" customHeight="1">
       <c r="A16" t="n">
@@ -3776,7 +3825,7 @@
       <c r="B16" t="n">
         <v>0</v>
       </c>
-      <c r="C16" s="9" t="inlineStr">
+      <c r="C16" s="6" t="inlineStr">
         <is>
           <t>SA</t>
         </is>
@@ -3838,7 +3887,7 @@
       </c>
       <c r="S16" s="1" t="inlineStr"/>
       <c r="T16" s="1" t="inlineStr"/>
-      <c r="U16" s="2" t="inlineStr"/>
+      <c r="U16" s="3" t="inlineStr"/>
       <c r="V16" s="1" t="inlineStr"/>
       <c r="W16" s="1" t="inlineStr"/>
       <c r="X16" s="1" t="inlineStr"/>
@@ -3957,6 +4006,9 @@
       <c r="BK16" t="n">
         <v>0</v>
       </c>
+      <c r="BL16" t="n">
+        <v>0</v>
+      </c>
     </row>
     <row r="17" ht="28" customHeight="1">
       <c r="A17" t="n">
@@ -3965,7 +4017,7 @@
       <c r="B17" t="n">
         <v>0</v>
       </c>
-      <c r="C17" s="9" t="inlineStr">
+      <c r="C17" s="6" t="inlineStr">
         <is>
           <t>VOR</t>
         </is>
@@ -4258,9 +4310,12 @@
       <c r="BK17" t="n">
         <v>0</v>
       </c>
+      <c r="BL17" t="n">
+        <v>0</v>
+      </c>
     </row>
   </sheetData>
-  <autoFilter ref="A1:BK17"/>
+  <autoFilter ref="A1:BL17"/>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
   <tableParts count="1">
     <tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="rId1"/>

</xml_diff>